<commit_message>
Added oligo probe panel: 10x Genomics; Xenium Prime 5K Mouse Pan Tissues & Pathways Panel, 2 rxns; PN 1000725
Closes #186
</commit_message>
<xml_diff>
--- a/xenium/latest/xenium.xlsx
+++ b/xenium/latest/xenium.xlsx
@@ -44,10 +44,10 @@
     </comment>
     <comment ref="B1" authorId="1">
       <text>
-        <t>A locally assigned identifier provided by the data provider for the dataset. It
-is used to reference an external metadata record that may be maintained
-independently, enabling traceability and supporting provenance tracking.
-Example: Visium_9OLC_A4_S1</t>
+        <t>An identifier assigned by the data provider to reference an external metadata
+record for the dataset. The external record may be maintained independently and
+can support dataset traceability and provenance tracking. Leave this field empty
+if no such identifier exists.</t>
       </text>
     </comment>
     <comment ref="C1" authorId="1">
@@ -289,7 +289,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="527" uniqueCount="506">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="523">
   <si>
     <t>parent_sample_id</t>
   </si>
@@ -303,94 +303,322 @@
     <t>dataset_type</t>
   </si>
   <si>
+    <t>Cell DIVE</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000159</t>
+  </si>
+  <si>
+    <t>CODEX</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000160</t>
+  </si>
+  <si>
+    <t>Light Sheet</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000168</t>
+  </si>
+  <si>
+    <t>MIBI</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000172</t>
+  </si>
+  <si>
+    <t>LC-MS</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000194</t>
+  </si>
+  <si>
     <t>HiFi-Slide</t>
   </si>
   <si>
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000195</t>
   </si>
   <si>
+    <t>Histology</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000197</t>
+  </si>
+  <si>
+    <t>PhenoCycler</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000199</t>
+  </si>
+  <si>
+    <t>CyCIF</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000200</t>
+  </si>
+  <si>
+    <t>MALDI</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000201</t>
+  </si>
+  <si>
+    <t>SIMS</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000202</t>
+  </si>
+  <si>
+    <t>DESI</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000204</t>
+  </si>
+  <si>
+    <t>Auto-fluorescence</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000205</t>
+  </si>
+  <si>
+    <t>Confocal</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000206</t>
+  </si>
+  <si>
+    <t>Thick section Multiphoton MxIF</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000207</t>
+  </si>
+  <si>
+    <t>Second Harmonic Generation (SHG)</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000208</t>
+  </si>
+  <si>
+    <t>Enhanced Stimulated Raman Spectroscopy (SRS)</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000209</t>
+  </si>
+  <si>
+    <t>10X Multiome</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000215</t>
+  </si>
+  <si>
+    <t>Molecular Cartography</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000217</t>
+  </si>
+  <si>
+    <t>CosMx Transcriptomics</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000218</t>
+  </si>
+  <si>
+    <t>Xenium</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000219</t>
+  </si>
+  <si>
+    <t>MERFISH</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000221</t>
+  </si>
+  <si>
     <t>SNARE-seq2</t>
   </si>
   <si>
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000264</t>
   </si>
   <si>
+    <t>2D Imaging Mass Cytometry</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000296</t>
+  </si>
+  <si>
+    <t>GeoMx (NGS)</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000300</t>
+  </si>
+  <si>
+    <t>GeoMx (nCounter)</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000301</t>
+  </si>
+  <si>
+    <t>Visium (no probes)</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000302</t>
+  </si>
+  <si>
+    <t>Visium (with probes)</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000303</t>
+  </si>
+  <si>
+    <t>ATACseq</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000309</t>
+  </si>
+  <si>
+    <t>RNAseq</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000310</t>
+  </si>
+  <si>
+    <t>RNAseq (with probes)</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000311</t>
+  </si>
+  <si>
+    <t>nanoSPLITS</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000312</t>
+  </si>
+  <si>
+    <t>MUSIC</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000328</t>
+  </si>
+  <si>
+    <t>Resolve</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000384</t>
+  </si>
+  <si>
+    <t>Stereo-seq</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000385</t>
+  </si>
+  <si>
+    <t>Seq-Scope</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000390</t>
+  </si>
+  <si>
+    <t>DART-FISH</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000396</t>
+  </si>
+  <si>
+    <t>seqFISH</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000397</t>
+  </si>
+  <si>
+    <t>MS Lipidomics</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000405</t>
+  </si>
+  <si>
+    <t>CyTOF</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000407</t>
+  </si>
+  <si>
+    <t>DBiT-seq</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000428</t>
+  </si>
+  <si>
+    <t>Singular Genomics G4X</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000429</t>
+  </si>
+  <si>
+    <t>CosMx Proteomics</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000435</t>
+  </si>
+  <si>
+    <t>FACS</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000440</t>
+  </si>
+  <si>
+    <t>Olink</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000441</t>
+  </si>
+  <si>
+    <t>4i</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000447</t>
+  </si>
+  <si>
+    <t>MPLEx</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000448</t>
+  </si>
+  <si>
+    <t>Pixel-seqV2</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000450</t>
+  </si>
+  <si>
+    <t>Visium HD</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000451</t>
+  </si>
+  <si>
     <t>COMET</t>
   </si>
   <si>
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000458</t>
   </si>
   <si>
-    <t>Visium (no probes)</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000302</t>
-  </si>
-  <si>
-    <t>DESI</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000204</t>
-  </si>
-  <si>
-    <t>Confocal</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000206</t>
-  </si>
-  <si>
-    <t>Stereo-seq</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000385</t>
-  </si>
-  <si>
-    <t>Visium (with probes)</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000303</t>
-  </si>
-  <si>
-    <t>Molecular Cartography</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000217</t>
-  </si>
-  <si>
     <t>Virtual Histology</t>
   </si>
   <si>
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000473</t>
   </si>
   <si>
-    <t>DBiT-seq</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000428</t>
-  </si>
-  <si>
-    <t>Seq-Scope</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000390</t>
-  </si>
-  <si>
-    <t>CosMx Transcriptomics</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000218</t>
-  </si>
-  <si>
-    <t>CyCIF</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000200</t>
-  </si>
-  <si>
-    <t>Light Sheet</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000168</t>
+    <t>Raman Imaging</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000475</t>
+  </si>
+  <si>
+    <t>STARmap</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000476</t>
   </si>
   <si>
     <t>iCLAP</t>
@@ -399,112 +627,16 @@
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000479</t>
   </si>
   <si>
-    <t>seqFISH</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000397</t>
-  </si>
-  <si>
-    <t>ATACseq</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000309</t>
-  </si>
-  <si>
-    <t>CosMx Proteomics</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000435</t>
-  </si>
-  <si>
-    <t>Singular Genomics G4X</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000429</t>
-  </si>
-  <si>
-    <t>Visium HD</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000451</t>
-  </si>
-  <si>
-    <t>MERFISH</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000221</t>
-  </si>
-  <si>
-    <t>10X Multiome</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000215</t>
-  </si>
-  <si>
-    <t>4i</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000447</t>
-  </si>
-  <si>
-    <t>PhenoCycler</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000199</t>
-  </si>
-  <si>
-    <t>Second Harmonic Generation (SHG)</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000208</t>
-  </si>
-  <si>
-    <t>Thick section Multiphoton MxIF</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000207</t>
-  </si>
-  <si>
     <t>MACSima</t>
   </si>
   <si>
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000480</t>
   </si>
   <si>
-    <t>CyTOF</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000407</t>
-  </si>
-  <si>
-    <t>Olink</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000441</t>
-  </si>
-  <si>
-    <t>MIBI</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000172</t>
-  </si>
-  <si>
-    <t>Auto-fluorescence</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000205</t>
-  </si>
-  <si>
-    <t>FACS</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000440</t>
-  </si>
-  <si>
-    <t>Xenium</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000219</t>
+    <t>Illumina Spatial ver0</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000487</t>
   </si>
   <si>
     <t>DNA Methylation</t>
@@ -513,157 +645,121 @@
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000490</t>
   </si>
   <si>
-    <t>SIMS</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000202</t>
-  </si>
-  <si>
-    <t>Cell DIVE</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000159</t>
-  </si>
-  <si>
-    <t>CODEX</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000160</t>
-  </si>
-  <si>
-    <t>GeoMx (NGS)</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000300</t>
-  </si>
-  <si>
-    <t>MUSIC</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000328</t>
-  </si>
-  <si>
-    <t>Pixel-seqV2</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000450</t>
-  </si>
-  <si>
-    <t>MALDI</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000201</t>
-  </si>
-  <si>
-    <t>2D Imaging Mass Cytometry</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000296</t>
-  </si>
-  <si>
-    <t>Histology</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000197</t>
-  </si>
-  <si>
-    <t>Enhanced Stimulated Raman Spectroscopy (SRS)</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000209</t>
-  </si>
-  <si>
-    <t>Illumina Spatial ver0</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000487</t>
-  </si>
-  <si>
-    <t>DART-FISH</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000396</t>
-  </si>
-  <si>
-    <t>Resolve</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000384</t>
-  </si>
-  <si>
-    <t>RNAseq</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000310</t>
-  </si>
-  <si>
-    <t>LC-MS</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000194</t>
-  </si>
-  <si>
-    <t>nanoSPLITS</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000312</t>
-  </si>
-  <si>
-    <t>GeoMx (nCounter)</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000301</t>
-  </si>
-  <si>
-    <t>Raman Imaging</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000475</t>
-  </si>
-  <si>
-    <t>RNAseq (with probes)</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000311</t>
-  </si>
-  <si>
-    <t>MS Lipidomics</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000405</t>
-  </si>
-  <si>
-    <t>STARmap</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000476</t>
-  </si>
-  <si>
-    <t>MPLEx</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000448</t>
+    <t>Paired-Tag</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000492</t>
+  </si>
+  <si>
+    <t>snm3C-seq</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000504</t>
   </si>
   <si>
     <t>analyte_class</t>
   </si>
   <si>
+    <t>Chromatin</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C13201</t>
+  </si>
+  <si>
+    <t>Collagen</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C16447</t>
+  </si>
+  <si>
+    <t>Protein</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C17021</t>
+  </si>
+  <si>
+    <t>DNA</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C449</t>
+  </si>
+  <si>
+    <t>Metabolite</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C61154</t>
+  </si>
+  <si>
+    <t>Lipid</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C616</t>
+  </si>
+  <si>
+    <t>Peptide</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C735</t>
+  </si>
+  <si>
+    <t>RNA</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C812</t>
+  </si>
+  <si>
+    <t>Polysaccharide</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/CHEBI_18154</t>
+  </si>
+  <si>
+    <t>Fluorochrome</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/CHEBI_51217</t>
+  </si>
+  <si>
+    <t>Endogenous fluorophore</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000131</t>
+  </si>
+  <si>
+    <t>Nucleic acid + protein</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000273</t>
+  </si>
+  <si>
     <t>DNA + RNA</t>
   </si>
   <si>
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000327</t>
   </si>
   <si>
-    <t>Nucleic acid + protein</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000273</t>
-  </si>
-  <si>
-    <t>Chromatin</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C13201</t>
+    <t>Saturated lipid</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000388</t>
+  </si>
+  <si>
+    <t>Unsaturated lipid</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000389</t>
+  </si>
+  <si>
+    <t>Lipid + metabolite</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000401</t>
+  </si>
+  <si>
+    <t>RNA + protein</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000474</t>
   </si>
   <si>
     <t>Lipid + metabolite + protein</t>
@@ -672,90 +768,6 @@
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000478</t>
   </si>
   <si>
-    <t>RNA + protein</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000474</t>
-  </si>
-  <si>
-    <t>RNA</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C812</t>
-  </si>
-  <si>
-    <t>Metabolite</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C61154</t>
-  </si>
-  <si>
-    <t>Unsaturated lipid</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000389</t>
-  </si>
-  <si>
-    <t>Lipid + metabolite</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000401</t>
-  </si>
-  <si>
-    <t>Saturated lipid</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000388</t>
-  </si>
-  <si>
-    <t>Lipid</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C616</t>
-  </si>
-  <si>
-    <t>Protein</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C17021</t>
-  </si>
-  <si>
-    <t>Fluorochrome</t>
-  </si>
-  <si>
-    <t>http://purl.obolibrary.org/obo/CHEBI_51217</t>
-  </si>
-  <si>
-    <t>Collagen</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C16447</t>
-  </si>
-  <si>
-    <t>DNA</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C449</t>
-  </si>
-  <si>
-    <t>Peptide</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C735</t>
-  </si>
-  <si>
-    <t>Polysaccharide</t>
-  </si>
-  <si>
-    <t>http://purl.obolibrary.org/obo/CHEBI_18154</t>
-  </si>
-  <si>
-    <t>Endogenous fluorophore</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000131</t>
-  </si>
-  <si>
     <t>is_targeted</t>
   </si>
   <si>
@@ -768,28 +780,175 @@
     <t>acquisition_instrument_vendor</t>
   </si>
   <si>
+    <t>In-House</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C126386</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_003899</t>
+  </si>
+  <si>
+    <t>Thermo Fisher Scientific</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_008452</t>
+  </si>
+  <si>
+    <t>Leica Microsystems</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_008960</t>
+  </si>
+  <si>
+    <t>Miltenyi Biotec</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_008984</t>
+  </si>
+  <si>
+    <t>Illumina</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_010233</t>
+  </si>
+  <si>
+    <t>Hamamatsu</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_017105</t>
+  </si>
+  <si>
+    <t>Bruker</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_017365</t>
+  </si>
+  <si>
+    <t>Cytiva</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023581</t>
+  </si>
+  <si>
+    <t>Leica Biosystems</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023603</t>
+  </si>
+  <si>
+    <t>Keyence</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023604</t>
+  </si>
+  <si>
+    <t>Ionpath</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023605</t>
+  </si>
+  <si>
+    <t>Standard BioTools (Fluidigm)</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023606</t>
+  </si>
+  <si>
+    <t>Zeiss Microscopy</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023607</t>
+  </si>
+  <si>
+    <t>Andor</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023609</t>
+  </si>
+  <si>
+    <t>Sciex</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023651</t>
+  </si>
+  <si>
+    <t>10x Genomics</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023672</t>
+  </si>
+  <si>
+    <t>Akoya Biosciences</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023774</t>
+  </si>
+  <si>
+    <t>Resolve Biosciences</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023911</t>
+  </si>
+  <si>
+    <t>NanoString</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023912</t>
+  </si>
+  <si>
+    <t>Waters</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024589</t>
+  </si>
+  <si>
+    <t>Evident Scientific (Olympus)</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024782</t>
+  </si>
+  <si>
     <t>BGI Genomics</t>
   </si>
   <si>
     <t>https://identifiers.org/RRID:SCR_024848</t>
   </si>
   <si>
-    <t>Cytiva</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023581</t>
-  </si>
-  <si>
-    <t>Thermo Fisher Scientific</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_008452</t>
-  </si>
-  <si>
-    <t>Zeiss Microscopy</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023607</t>
+    <t>Motic</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024856</t>
+  </si>
+  <si>
+    <t>Huron Digital Pathology</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024996</t>
+  </si>
+  <si>
+    <t>GE Healthcare</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_025461</t>
+  </si>
+  <si>
+    <t>Vizgen</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026274</t>
+  </si>
+  <si>
+    <t>Element Biosciences</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026453</t>
+  </si>
+  <si>
+    <t>Singular Genomics</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026683</t>
   </si>
   <si>
     <t>Complete Genomics</t>
@@ -804,130 +963,16 @@
     <t>https://identifiers.org/RRID:SCR_027042</t>
   </si>
   <si>
-    <t>GE Healthcare</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_025461</t>
-  </si>
-  <si>
-    <t>Leica Microsystems</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_008960</t>
-  </si>
-  <si>
-    <t>Akoya Biosciences</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023774</t>
-  </si>
-  <si>
-    <t>NanoString</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023912</t>
-  </si>
-  <si>
-    <t>Element Biosciences</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_026453</t>
-  </si>
-  <si>
-    <t>Andor</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023609</t>
-  </si>
-  <si>
-    <t>Huron Digital Pathology</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_024996</t>
-  </si>
-  <si>
-    <t>Illumina</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_010233</t>
-  </si>
-  <si>
-    <t>Ionpath</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023605</t>
-  </si>
-  <si>
-    <t>Waters</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_024589</t>
-  </si>
-  <si>
-    <t>In-House</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C126386</t>
-  </si>
-  <si>
-    <t>Resolve Biosciences</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023911</t>
-  </si>
-  <si>
-    <t>Singular Genomics</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_026683</t>
-  </si>
-  <si>
-    <t>Vizgen</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_026274</t>
-  </si>
-  <si>
-    <t>Standard BioTools (Fluidigm)</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023606</t>
-  </si>
-  <si>
-    <t>Sciex</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023651</t>
-  </si>
-  <si>
-    <t>Bruker</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_017365</t>
-  </si>
-  <si>
-    <t>Evident Scientific (Olympus)</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_024782</t>
-  </si>
-  <si>
-    <t>Keyence</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023604</t>
-  </si>
-  <si>
-    <t>Miltenyi Biotec</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_008984</t>
-  </si>
-  <si>
-    <t>Leica Biosystems</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023603</t>
+    <t>Cytek Biosciences</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027071</t>
+  </si>
+  <si>
+    <t>Microscopes International</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027094</t>
   </si>
   <si>
     <t>Revvity</t>
@@ -936,55 +981,313 @@
     <t>https://identifiers.org/RRID:SCR_027779</t>
   </si>
   <si>
-    <t>Cytek Biosciences</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_027071</t>
-  </si>
-  <si>
-    <t>10x Genomics</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023672</t>
-  </si>
-  <si>
-    <t>Microscopes International</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_027094</t>
-  </si>
-  <si>
-    <t>Hamamatsu</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_017105</t>
-  </si>
-  <si>
-    <t>Motic</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_024856</t>
+    <t>MGI Tech</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_029020</t>
   </si>
   <si>
     <t>acquisition_instrument_model</t>
   </si>
   <si>
+    <t>Unknown</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C17998</t>
+  </si>
+  <si>
+    <t>Not applicable</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C48660</t>
+  </si>
+  <si>
+    <t>NextSeq 500</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_014983</t>
+  </si>
+  <si>
+    <t>NextSeq 550</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_016381</t>
+  </si>
+  <si>
+    <t>HiSeq 2500</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_016383</t>
+  </si>
+  <si>
+    <t>HiSeq 4000</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_016386</t>
+  </si>
+  <si>
+    <t>NovaSeq 6000</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_016387</t>
+  </si>
+  <si>
+    <t>iScan System</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_016388</t>
+  </si>
+  <si>
+    <t>BZ-X710</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_017202</t>
+  </si>
+  <si>
+    <t>LSM 710 Confocal Microscope</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_018063</t>
+  </si>
+  <si>
+    <t>Helios</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_019916</t>
+  </si>
+  <si>
+    <t>QTRAP 5500</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_020517</t>
+  </si>
+  <si>
+    <t>Q Exactive HF</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_020558</t>
+  </si>
+  <si>
+    <t>Orbitrap Fusion Tribrid</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_020559</t>
+  </si>
+  <si>
+    <t>Orbitrap Fusion Lumos Tribrid</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_020562</t>
+  </si>
+  <si>
+    <t>Q Exactive HF-X</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_020564</t>
+  </si>
+  <si>
+    <t>Q Exactive</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_020565</t>
+  </si>
+  <si>
+    <t>Q Exactive UHMR</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_020571</t>
+  </si>
+  <si>
+    <t>Zeiss LightSheet Z.1</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_020919</t>
+  </si>
+  <si>
+    <t>Axio Scan.Z1</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_020927</t>
+  </si>
+  <si>
+    <t>Aperio AT2</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_021256</t>
+  </si>
+  <si>
+    <t>NanoZoomer 2.0-HT</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_021658</t>
+  </si>
+  <si>
+    <t>Digital Spatial Profiler</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_021660</t>
+  </si>
+  <si>
+    <t>Biomark HD</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_022658</t>
+  </si>
+  <si>
+    <t>Hyperion Imaging System</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023195</t>
+  </si>
+  <si>
+    <t>PhenoImager Fusion</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023274</t>
+  </si>
+  <si>
+    <t>Zyla 4.2 sCMOS</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023610</t>
+  </si>
+  <si>
     <t>SCN400</t>
   </si>
   <si>
     <t>https://identifiers.org/RRID:SCR_023611</t>
   </si>
   <si>
+    <t>MIBIscope</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023613</t>
+  </si>
+  <si>
+    <t>NextSeq 2000</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023614</t>
+  </si>
+  <si>
+    <t>timsTOF FleX MALDI-2</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023615</t>
+  </si>
+  <si>
+    <t>IN Cell Analyzer 2200</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023616</t>
+  </si>
+  <si>
+    <t>BZ-X800</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023617</t>
+  </si>
+  <si>
+    <t>Orbitrap Eclipse Tribrid</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023618</t>
+  </si>
+  <si>
+    <t>Axio Observer 5</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023692</t>
+  </si>
+  <si>
+    <t>Axio Observer 3</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023693</t>
+  </si>
+  <si>
+    <t>Axio Observer 7</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023694</t>
+  </si>
+  <si>
+    <t>NanoZoomer S210</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023760</t>
+  </si>
+  <si>
+    <t>NanoZoomer S360</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023761</t>
+  </si>
+  <si>
+    <t>NanoZoomer S60</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023762</t>
+  </si>
+  <si>
+    <t>NanoZoomer-SQ</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023763</t>
+  </si>
+  <si>
+    <t>Phenocycler-Fusion 2.0</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023773</t>
+  </si>
+  <si>
+    <t>CosMx Spatial Molecular Imager</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023909</t>
+  </si>
+  <si>
+    <t>Xenium Analyzer</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023910</t>
+  </si>
+  <si>
+    <t>Lightsheet 7</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024448</t>
+  </si>
+  <si>
+    <t>Resolve Biosciences Molecular Cartography</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024449</t>
+  </si>
+  <si>
+    <t>NovaSeq X Plus</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024568</t>
+  </si>
+  <si>
+    <t>NovaSeq X</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024569</t>
+  </si>
+  <si>
     <t>STELLARIS 5</t>
   </si>
   <si>
     <t>https://identifiers.org/RRID:SCR_024663</t>
   </si>
   <si>
-    <t>BZ-X710</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_017202</t>
+    <t>VS200 Slide Scanner</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024783</t>
   </si>
   <si>
     <t>Pannoramic MIDI II Digital Scanner</t>
@@ -993,10 +1296,10 @@
     <t>https://identifiers.org/RRID:SCR_024834</t>
   </si>
   <si>
-    <t>Not applicable</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C48660</t>
+    <t>DNBSEQ-T7</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024847</t>
   </si>
   <si>
     <t>MoticEasyScan One</t>
@@ -1005,28 +1308,64 @@
     <t>https://identifiers.org/RRID:SCR_024855</t>
   </si>
   <si>
+    <t>DM6 B</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024857</t>
+  </si>
+  <si>
+    <t>TissueScope LE Slide Scanner</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024995</t>
+  </si>
+  <si>
     <t>EVOS M7000</t>
   </si>
   <si>
     <t>https://identifiers.org/RRID:SCR_025070</t>
   </si>
   <si>
-    <t>NovaSeq X</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_024569</t>
-  </si>
-  <si>
-    <t>LSM 710 Confocal Microscope</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_018063</t>
-  </si>
-  <si>
-    <t>NanoZoomer 2.0-HT</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_021658</t>
+    <t>Aperio CS2</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_025111</t>
+  </si>
+  <si>
+    <t>BZ-X810</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_025160</t>
+  </si>
+  <si>
+    <t>MERSCOPE Ultra</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026273</t>
+  </si>
+  <si>
+    <t>CyTOF XT</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026344</t>
+  </si>
+  <si>
+    <t>AVITI</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026452</t>
+  </si>
+  <si>
+    <t>SYNAPT XS</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026524</t>
+  </si>
+  <si>
+    <t>timsTOF Ultra</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026540</t>
   </si>
   <si>
     <t>timsTOF Ultra 2</t>
@@ -1035,10 +1374,133 @@
     <t>https://identifiers.org/RRID:SCR_026541</t>
   </si>
   <si>
-    <t>Lightsheet 7</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_024448</t>
+    <t>timsTOF SCP</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026542</t>
+  </si>
+  <si>
+    <t>timsTOF HT</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026543</t>
+  </si>
+  <si>
+    <t>timsTOF Pro</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026544</t>
+  </si>
+  <si>
+    <t>timsTOF Pro 2</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026545</t>
+  </si>
+  <si>
+    <t>CyTOF 2</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026551</t>
+  </si>
+  <si>
+    <t>DMi8</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026672</t>
+  </si>
+  <si>
+    <t>G4X Spatial Sequencer</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026684</t>
+  </si>
+  <si>
+    <t>timsTOF FleX</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026925</t>
+  </si>
+  <si>
+    <t>Cytek Northern Lights</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027072</t>
+  </si>
+  <si>
+    <t>Axio Zoom.V16</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027090</t>
+  </si>
+  <si>
+    <t>solariX</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027095</t>
+  </si>
+  <si>
+    <t>uScopeHXII-20</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027101</t>
+  </si>
+  <si>
+    <t>Juno System</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027198</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027323</t>
+  </si>
+  <si>
+    <t>Panoramic 150 Digital Scanner</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027467</t>
+  </si>
+  <si>
+    <t>Opera Phenix Plus HCS</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027780</t>
+  </si>
+  <si>
+    <t>SYNAPT G2-Si</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027782</t>
+  </si>
+  <si>
+    <t>Opera Phenix HCS</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027817</t>
+  </si>
+  <si>
+    <t>MACSima System</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027923</t>
+  </si>
+  <si>
+    <t>NanoZoomer 2.0-RS</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_028001</t>
+  </si>
+  <si>
+    <t>Orbitrap Astral</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_028684</t>
+  </si>
+  <si>
+    <t>Olink Signature Q100</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_028906</t>
   </si>
   <si>
     <t>Phenocycler-Fusion 1.0</t>
@@ -1047,274 +1509,16 @@
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000316</t>
   </si>
   <si>
-    <t>DNBSEQ-T7</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_024847</t>
-  </si>
-  <si>
-    <t>timsTOF Pro</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_026544</t>
-  </si>
-  <si>
-    <t>Unknown</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C17998</t>
-  </si>
-  <si>
-    <t>AVITI</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_026452</t>
-  </si>
-  <si>
-    <t>DMi8</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_026672</t>
-  </si>
-  <si>
-    <t>Opera Phenix Plus HCS</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_027780</t>
-  </si>
-  <si>
-    <t>timsTOF Pro 2</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_026545</t>
-  </si>
-  <si>
-    <t>Q Exactive UHMR</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_020571</t>
-  </si>
-  <si>
-    <t>Q Exactive</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_020565</t>
-  </si>
-  <si>
-    <t>timsTOF SCP</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_026542</t>
-  </si>
-  <si>
-    <t>Zyla 4.2 sCMOS</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023610</t>
-  </si>
-  <si>
-    <t>Helios</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_019916</t>
-  </si>
-  <si>
-    <t>uScopeHXII-20</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_027101</t>
-  </si>
-  <si>
-    <t>Orbitrap Fusion Tribrid</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_020559</t>
-  </si>
-  <si>
     <t>Custom: Multiphoton</t>
   </si>
   <si>
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000317</t>
   </si>
   <si>
-    <t>QTRAP 5500</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_020517</t>
-  </si>
-  <si>
-    <t>timsTOF Ultra</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_026540</t>
-  </si>
-  <si>
-    <t>BZ-X800</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023617</t>
-  </si>
-  <si>
-    <t>CyTOF 2</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_026551</t>
-  </si>
-  <si>
-    <t>G4X Spatial Sequencer</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_026684</t>
-  </si>
-  <si>
-    <t>NextSeq 500</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_014983</t>
-  </si>
-  <si>
-    <t>NanoZoomer S360</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023761</t>
-  </si>
-  <si>
-    <t>Hyperion Imaging System</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023195</t>
-  </si>
-  <si>
-    <t>NovaSeq X Plus</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_024568</t>
-  </si>
-  <si>
-    <t>CyTOF XT</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_026344</t>
-  </si>
-  <si>
-    <t>NanoZoomer-SQ</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023763</t>
-  </si>
-  <si>
-    <t>NextSeq 550</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_016381</t>
-  </si>
-  <si>
-    <t>Axio Zoom.V16</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_027090</t>
-  </si>
-  <si>
-    <t>Digital Spatial Profiler</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_021660</t>
-  </si>
-  <si>
-    <t>timsTOF FleX</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_026925</t>
-  </si>
-  <si>
-    <t>timsTOF FleX MALDI-2</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023615</t>
-  </si>
-  <si>
-    <t>NanoZoomer S210</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023760</t>
-  </si>
-  <si>
-    <t>BZ-X810</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_025160</t>
-  </si>
-  <si>
-    <t>Axio Observer 7</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023694</t>
-  </si>
-  <si>
-    <t>Cytek Northern Lights</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_027072</t>
-  </si>
-  <si>
-    <t>Opera Phenix HCS</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_027817</t>
-  </si>
-  <si>
-    <t>Zeiss LightSheet Z.1</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_020919</t>
-  </si>
-  <si>
-    <t>IN Cell Analyzer 2200</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023616</t>
-  </si>
-  <si>
-    <t>timsTOF HT</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_026543</t>
-  </si>
-  <si>
-    <t>PhenoImager Fusion</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023274</t>
-  </si>
-  <si>
-    <t>DM6 B</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_024857</t>
-  </si>
-  <si>
-    <t>Phenocycler-Fusion 2.0</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023773</t>
-  </si>
-  <si>
-    <t>Aperio CS2</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_025111</t>
-  </si>
-  <si>
-    <t>Orbitrap Fusion Lumos Tribrid</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_020562</t>
-  </si>
-  <si>
-    <t>Resolve Biosciences Molecular Cartography</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_024449</t>
+    <t>MERSCOPE</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000404</t>
   </si>
   <si>
     <t>MALDI timsTOF Flex Prototype</t>
@@ -1323,177 +1527,30 @@
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000433</t>
   </si>
   <si>
-    <t>TissueScope LE Slide Scanner</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_024995</t>
-  </si>
-  <si>
-    <t>VS200 Slide Scanner</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_024783</t>
-  </si>
-  <si>
-    <t>Axio Observer 5</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023692</t>
-  </si>
-  <si>
-    <t>NanoZoomer 2.0-RS</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_028001</t>
-  </si>
-  <si>
-    <t>Axio Observer 3</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023693</t>
-  </si>
-  <si>
-    <t>HiSeq 2500</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_016383</t>
-  </si>
-  <si>
-    <t>Orbitrap Eclipse Tribrid</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023618</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_027323</t>
-  </si>
-  <si>
-    <t>MERSCOPE</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000404</t>
-  </si>
-  <si>
-    <t>NextSeq 2000</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023614</t>
-  </si>
-  <si>
-    <t>NovaSeq 6000</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_016387</t>
-  </si>
-  <si>
-    <t>HiSeq 4000</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_016386</t>
-  </si>
-  <si>
-    <t>Q Exactive HF-X</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_020564</t>
-  </si>
-  <si>
-    <t>solariX</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_027095</t>
-  </si>
-  <si>
-    <t>Panoramic 150 Digital Scanner</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_027467</t>
-  </si>
-  <si>
-    <t>Aperio AT2</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_021256</t>
-  </si>
-  <si>
-    <t>MIBIscope</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023613</t>
-  </si>
-  <si>
-    <t>SYNAPT G2-Si</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_027782</t>
-  </si>
-  <si>
-    <t>MACSima System</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_027923</t>
-  </si>
-  <si>
-    <t>Biomark HD</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_022658</t>
-  </si>
-  <si>
-    <t>NanoZoomer S60</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023762</t>
-  </si>
-  <si>
-    <t>CosMx Spatial Molecular Imager</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023909</t>
-  </si>
-  <si>
-    <t>MERSCOPE Ultra</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_026273</t>
-  </si>
-  <si>
-    <t>Axio Scan.Z1</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_020927</t>
-  </si>
-  <si>
-    <t>Juno System</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_027198</t>
-  </si>
-  <si>
-    <t>Q Exactive HF</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_020558</t>
-  </si>
-  <si>
-    <t>Xenium Analyzer</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023910</t>
-  </si>
-  <si>
     <t>source_storage_duration_value</t>
   </si>
   <si>
     <t>source_storage_duration_unit</t>
   </si>
   <si>
+    <t>minute</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/UO_0000031</t>
+  </si>
+  <si>
     <t>hour</t>
   </si>
   <si>
     <t>http://purl.obolibrary.org/obo/UO_0000032</t>
   </si>
   <si>
+    <t>day</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/UO_0000033</t>
+  </si>
+  <si>
     <t>month</t>
   </si>
   <si>
@@ -1506,18 +1563,6 @@
     <t>http://purl.obolibrary.org/obo/UO_0000036</t>
   </si>
   <si>
-    <t>day</t>
-  </si>
-  <si>
-    <t>http://purl.obolibrary.org/obo/UO_0000033</t>
-  </si>
-  <si>
-    <t>minute</t>
-  </si>
-  <si>
-    <t>http://purl.obolibrary.org/obo/UO_0000031</t>
-  </si>
-  <si>
     <t>time_since_acquisition_instrument_calibration_value</t>
   </si>
   <si>
@@ -1578,22 +1623,106 @@
     <t>oligo_probe_panel</t>
   </si>
   <si>
+    <t>Custom</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C65167</t>
+  </si>
+  <si>
+    <t>10x Genomics; Visium Human Transcriptome Probe Kit v2 - Small; PN 1000466</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000274</t>
+  </si>
+  <si>
+    <t>10x Genomics; Chromium Fixed RNA Kit, Human Transcriptome, 4 rxns x 1 BC; PN 1000474</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000306</t>
+  </si>
+  <si>
+    <t>10x Genomics; Visium Human Transcriptome Probe Kit-Small; PN 1000363</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000326</t>
+  </si>
+  <si>
+    <t>10x Genomics; Visium Mouse Transcriptome Probe Kit - Small; PN 1000365</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000362</t>
+  </si>
+  <si>
+    <t>NanoString Technologies; GeoMx Human Whole Transcriptome Atlas, 4 slides; PN GMX-RNA-NGS-HuWTA-4</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000363</t>
+  </si>
+  <si>
+    <t>NanoString Technologies; GeoMx Mouse Whole Transcriptome Atlas, 4 slides; PN GMX-RNA-NGS-MsWTA-4</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000364</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Next GEM Single Cell Fixed RNA Human Transcriptome Probe Kit, 64 rxns; PN 1000456</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000376</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Next GEM Single Cell Fixed RNA Human Transcriptome Probe Kit, 16 rxns; PN 1000420</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000382</t>
+  </si>
+  <si>
+    <t>10x Genomics; Visium Human Transcriptome Probe Kit-Large; PN 1000364</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000383</t>
+  </si>
+  <si>
     <t>10x Genomics; Chromium Next GEM Single Cell Fixed RNA Mouse Transcriptome Probe Kit, 64 rxns; PN 1000492</t>
   </si>
   <si>
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000393</t>
   </si>
   <si>
+    <t>10x Genomics; Xenium Human Multi-Tissue and Cancer Panel v1; PN 1000626</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000395</t>
+  </si>
+  <si>
     <t>10x Genomics; Xenium Prime 5K Human Pan Tissue &amp; Pathways Panel; PN 1000724</t>
   </si>
   <si>
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000426</t>
   </si>
   <si>
-    <t>10x Genomics; Visium Human Transcriptome Probe Kit-Large; PN 1000364</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000383</t>
+    <t>NanoString Technologies; CosMx Human Universal Cell Characterization Panel (RNA, 1000 Plex); PN CMX-H-USCP-1KP-R</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000430</t>
+  </si>
+  <si>
+    <t>10x Genomics; Visium Mouse Transcriptome Probe Kit v2.0 - Small; PN 1000667</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000431</t>
+  </si>
+  <si>
+    <t>NanoString Technologies; CosMx Human Immuno-Oncology Panel (Protein, 64 Plex); PN CMX-H-IOP-64P-P</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000436</t>
+  </si>
+  <si>
+    <t>NanoString Technologies; CosMx Mouse Neuroscience Panel (Protein, 64 Plex); PN CMX-M-Neuro-64P-P</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000437</t>
   </si>
   <si>
     <t>10x Genomics; Xenium Mouse Multi-Tissue Atlassing Panel; PN 1000627</t>
@@ -1602,166 +1731,88 @@
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000442</t>
   </si>
   <si>
+    <t>10x Genomics; Xenium Human Lung Gene Expression Panel; PN 1000601</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000443</t>
+  </si>
+  <si>
+    <t>10x Genomics; Xenium Custom Gene Expression Panel (51-100 genes); PN 1000561</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000444</t>
+  </si>
+  <si>
+    <t>10x Genomics; Xenium Custom Gene Expression Panel (up to 50 genes); PN 1000464</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000445</t>
+  </si>
+  <si>
+    <t>10x Genomics; Xenium Human Colon Gene Expression Panel; PN 1000642</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000446</t>
+  </si>
+  <si>
+    <t>NanoString Technologies; CosMx Mouse Neuroscience Panel (RNA, 1000 Plex); PN CMX-M-NEUP-R</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000452</t>
+  </si>
+  <si>
+    <t>NanoString Technologies; CosMx Hs WTX RNA Panel Kit, 2 slides: PN 121500047</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000453</t>
+  </si>
+  <si>
+    <t>NanoString Technologies; CosMx Hs Univ Cell (RNA, 1000 Plex); PN 121500002</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000454</t>
+  </si>
+  <si>
+    <t>NanoString Technologies; CosMx Human 6K Discovery Panel (RNA, 6175 Plex); PN 121500041</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000455</t>
+  </si>
+  <si>
+    <t>NanoString Technologies; CosMx Mouse Universal Cell Characterization Panel (RNA, 1000 Plex); PN CMX-M-USCP-1KP-R</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000457</t>
+  </si>
+  <si>
+    <t>10x Genomics; Chromium Fixed RNA Kit, Human Transcriptome 16 rxns x 16 BC; PN 1000547</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000477</t>
+  </si>
+  <si>
     <t>10x Genomics; GEM-X Flex Human Transcriptome Probe Kit, 16 samples; PN 1000785</t>
   </si>
   <si>
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000481</t>
   </si>
   <si>
-    <t>10x Genomics; Visium Human Transcriptome Probe Kit-Small; PN 1000363</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000326</t>
-  </si>
-  <si>
-    <t>10x Genomics; Visium Mouse Transcriptome Probe Kit v2.0 - Small; PN 1000667</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000431</t>
-  </si>
-  <si>
     <t>NanoString Technologies; GeoMx Human IO Proteome Atlas, 4 slides; PN 121300160</t>
   </si>
   <si>
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000488</t>
   </si>
   <si>
-    <t>10x Genomics; Visium Human Transcriptome Probe Kit v2 - Small; PN 1000466</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000274</t>
-  </si>
-  <si>
-    <t>NanoString Technologies; CosMx Human 6K Discovery Panel (RNA, 6175 Plex); PN 121500041</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000455</t>
-  </si>
-  <si>
-    <t>NanoString Technologies; CosMx Mouse Universal Cell Characterization Panel (RNA, 1000 Plex); PN CMX-M-USCP-1KP-R</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000457</t>
-  </si>
-  <si>
-    <t>10x Genomics; Xenium Custom Gene Expression Panel (51-100 genes); PN 1000561</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000444</t>
-  </si>
-  <si>
-    <t>10X Genomics; Chromium Next GEM Single Cell Fixed RNA Human Transcriptome Probe Kit, 64 rxns; PN 1000456</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000376</t>
-  </si>
-  <si>
-    <t>10x Genomics; Xenium Human Colon Gene Expression Panel; PN 1000642</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000446</t>
-  </si>
-  <si>
-    <t>NanoString Technologies; CosMx Human Immuno-Oncology Panel (Protein, 64 Plex); PN CMX-H-IOP-64P-P</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000436</t>
-  </si>
-  <si>
-    <t>10x Genomics; Chromium Fixed RNA Kit, Human Transcriptome 16 rxns x 16 BC; PN 1000547</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000477</t>
-  </si>
-  <si>
-    <t>10x Genomics; Visium Mouse Transcriptome Probe Kit - Small; PN 1000365</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000362</t>
-  </si>
-  <si>
-    <t>NanoString Technologies; CosMx Hs WTX RNA Panel Kit, 2 slides: PN 121500047</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000453</t>
-  </si>
-  <si>
-    <t>10x Genomics; Xenium Human Lung Gene Expression Panel; PN 1000601</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000443</t>
-  </si>
-  <si>
-    <t>NanoString Technologies; CosMx Mouse Neuroscience Panel (Protein, 64 Plex); PN CMX-M-Neuro-64P-P</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000437</t>
-  </si>
-  <si>
-    <t>NanoString Technologies; GeoMx Mouse Whole Transcriptome Atlas, 4 slides; PN GMX-RNA-NGS-MsWTA-4</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000364</t>
-  </si>
-  <si>
-    <t>NanoString Technologies; CosMx Mouse Neuroscience Panel (RNA, 1000 Plex); PN CMX-M-NEUP-R</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000452</t>
-  </si>
-  <si>
-    <t>Custom</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C65167</t>
-  </si>
-  <si>
-    <t>NanoString Technologies; GeoMx Human Whole Transcriptome Atlas, 4 slides; PN GMX-RNA-NGS-HuWTA-4</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000363</t>
-  </si>
-  <si>
-    <t>10x Genomics; Xenium Human Multi-Tissue and Cancer Panel v1; PN 1000626</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000395</t>
-  </si>
-  <si>
-    <t>10x Genomics; Xenium Custom Gene Expression Panel (up to 50 genes); PN 1000464</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000445</t>
-  </si>
-  <si>
-    <t>10x Genomics; Chromium Fixed RNA Kit, Human Transcriptome, 4 rxns x 1 BC; PN 1000474</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000306</t>
-  </si>
-  <si>
     <t>10x Genomics; Xenium Human Skin Gene Expression Panel; PN 1000643</t>
   </si>
   <si>
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000491</t>
   </si>
   <si>
-    <t>NanoString Technologies; CosMx Human Universal Cell Characterization Panel (RNA, 1000 Plex); PN CMX-H-USCP-1KP-R</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000430</t>
-  </si>
-  <si>
-    <t>10X Genomics; Chromium Next GEM Single Cell Fixed RNA Human Transcriptome Probe Kit, 16 rxns; PN 1000420</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000382</t>
-  </si>
-  <si>
-    <t>NanoString Technologies; CosMx Hs Univ Cell (RNA, 1000 Plex); PN 121500002</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000454</t>
+    <t>10x Genomics; Xenium Prime 5K Mouse Pan Tissues &amp; Pathways Panel, 2 rxns; PN 1000725</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000506</t>
   </si>
   <si>
     <t>is_custom_probes_used</t>
@@ -1800,7 +1851,7 @@
     <t>pav:createdOn</t>
   </si>
   <si>
-    <t>2026-06-11T13:20:33-07:00</t>
+    <t>2026-10-20T13:27:42-07:00</t>
   </si>
   <si>
     <t>pav:derivedFrom</t>
@@ -1959,105 +2010,105 @@
         <v>3</v>
       </c>
       <c r="E1" t="s" s="1">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="F1" t="s" s="1">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="G1" t="s" s="1">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="H1" t="s" s="1">
-        <v>225</v>
+        <v>232</v>
       </c>
       <c r="I1" t="s" s="1">
-        <v>397</v>
+        <v>412</v>
       </c>
       <c r="J1" t="s" s="1">
-        <v>398</v>
+        <v>413</v>
       </c>
       <c r="K1" t="s" s="1">
-        <v>409</v>
+        <v>424</v>
       </c>
       <c r="L1" t="s" s="1">
-        <v>410</v>
+        <v>425</v>
       </c>
       <c r="M1" t="s" s="1">
-        <v>411</v>
+        <v>426</v>
       </c>
       <c r="N1" t="s" s="1">
-        <v>412</v>
+        <v>427</v>
       </c>
       <c r="O1" t="s" s="1">
-        <v>413</v>
+        <v>428</v>
       </c>
       <c r="P1" t="s" s="1">
-        <v>414</v>
+        <v>429</v>
       </c>
       <c r="Q1" t="s" s="1">
-        <v>419</v>
+        <v>434</v>
       </c>
       <c r="R1" t="s" s="1">
-        <v>420</v>
+        <v>435</v>
       </c>
       <c r="S1" t="s" s="1">
-        <v>421</v>
+        <v>436</v>
       </c>
       <c r="T1" t="s" s="1">
-        <v>422</v>
+        <v>437</v>
       </c>
       <c r="U1" t="s" s="1">
-        <v>423</v>
+        <v>438</v>
       </c>
       <c r="V1" t="s" s="1">
-        <v>424</v>
+        <v>439</v>
       </c>
       <c r="W1" t="s" s="1">
-        <v>425</v>
+        <v>440</v>
       </c>
       <c r="X1" t="s" s="1">
-        <v>426</v>
+        <v>441</v>
       </c>
       <c r="Y1" t="s" s="1">
-        <v>427</v>
+        <v>442</v>
       </c>
       <c r="Z1" t="s" s="1">
-        <v>428</v>
+        <v>443</v>
       </c>
       <c r="AA1" t="s" s="1">
-        <v>491</v>
+        <v>508</v>
       </c>
       <c r="AB1" t="s" s="1">
-        <v>492</v>
+        <v>509</v>
       </c>
       <c r="AC1" t="s" s="1">
-        <v>493</v>
+        <v>510</v>
       </c>
       <c r="AD1" t="s" s="1">
-        <v>494</v>
+        <v>511</v>
       </c>
       <c r="AE1" t="s" s="1">
-        <v>495</v>
+        <v>512</v>
       </c>
       <c r="AF1" t="s" s="1">
-        <v>496</v>
+        <v>513</v>
       </c>
       <c r="AG1" t="s" s="1">
-        <v>497</v>
+        <v>514</v>
       </c>
     </row>
     <row r="2">
       <c r="D2" t="s" s="5">
-        <v>70</v>
+        <v>44</v>
       </c>
       <c r="AG2" t="s" s="34">
-        <v>498</v>
+        <v>515</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="22">
     <dataValidation type="list" sqref="D2:D1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
-      <formula1>'dataset_type'!$A$1:$A$57</formula1>
+      <formula1>'dataset_type'!$A$1:$A$59</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="E2:E1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
       <formula1>'analyte_class'!$A$1:$A$18</formula1>
@@ -2066,10 +2117,10 @@
       <formula1>'is_targeted'!$A$1:$A$2</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="G2:G1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
-      <formula1>'acquisition_instrument_vendor'!$A$1:$A$33</formula1>
+      <formula1>'acquisition_instrument_vendor'!$A$1:$A$35</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="H2:H1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
-      <formula1>'acquisition_instrument_model'!$A$1:$A$87</formula1>
+      <formula1>'acquisition_instrument_model'!$A$1:$A$91</formula1>
     </dataValidation>
     <dataValidation type="decimal" operator="greaterThanOrEqual" sqref="I2:I1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be greater than 0" showErrorMessage="true">
       <formula1>0</formula1>
@@ -2122,7 +2173,7 @@
       <formula1>'probe_hybridization_time_unit'!$A$1:$A$2</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="Z2:Z1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
-      <formula1>'oligo_probe_panel'!$A$1:$A$31</formula1>
+      <formula1>'oligo_probe_panel'!$A$1:$A$32</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="AA2:AA1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
       <formula1>'is_custom_probes_used'!$A$1:$A$2</formula1>
@@ -2145,10 +2196,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>407</v>
+        <v>414</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>408</v>
+        <v>415</v>
       </c>
     </row>
   </sheetData>
@@ -2163,10 +2214,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>407</v>
+        <v>414</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>408</v>
+        <v>415</v>
       </c>
     </row>
   </sheetData>
@@ -2181,18 +2232,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>399</v>
+        <v>414</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>400</v>
+        <v>415</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>407</v>
+        <v>416</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>408</v>
+        <v>417</v>
       </c>
     </row>
   </sheetData>
@@ -2202,255 +2253,263 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:B32"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>429</v>
+        <v>444</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>430</v>
+        <v>445</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>431</v>
+        <v>446</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>432</v>
+        <v>447</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>433</v>
+        <v>448</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>434</v>
+        <v>449</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>435</v>
+        <v>450</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>436</v>
+        <v>451</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>437</v>
+        <v>452</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>438</v>
+        <v>453</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>439</v>
+        <v>454</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>440</v>
+        <v>455</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>441</v>
+        <v>456</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>442</v>
+        <v>457</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>443</v>
+        <v>458</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>444</v>
+        <v>459</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>445</v>
+        <v>460</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>446</v>
+        <v>461</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>447</v>
+        <v>462</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>448</v>
+        <v>463</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>449</v>
+        <v>464</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>450</v>
+        <v>465</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>451</v>
+        <v>466</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>452</v>
+        <v>467</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>453</v>
+        <v>468</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>454</v>
+        <v>469</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>455</v>
+        <v>470</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>456</v>
+        <v>471</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>457</v>
+        <v>472</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>458</v>
+        <v>473</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>459</v>
+        <v>474</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>460</v>
+        <v>475</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>461</v>
+        <v>476</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>462</v>
+        <v>477</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>463</v>
+        <v>478</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>464</v>
+        <v>479</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
-        <v>465</v>
+        <v>480</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>466</v>
+        <v>481</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="0">
-        <v>467</v>
+        <v>482</v>
       </c>
       <c r="B20" t="s" s="0">
-        <v>468</v>
+        <v>483</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="0">
-        <v>469</v>
+        <v>484</v>
       </c>
       <c r="B21" t="s" s="0">
-        <v>470</v>
+        <v>485</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
-        <v>471</v>
+        <v>486</v>
       </c>
       <c r="B22" t="s" s="0">
-        <v>472</v>
+        <v>487</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
-        <v>473</v>
+        <v>488</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>474</v>
+        <v>489</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="0">
-        <v>475</v>
+        <v>490</v>
       </c>
       <c r="B24" t="s" s="0">
-        <v>476</v>
+        <v>491</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="0">
-        <v>477</v>
+        <v>492</v>
       </c>
       <c r="B25" t="s" s="0">
-        <v>478</v>
+        <v>493</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="0">
-        <v>479</v>
+        <v>494</v>
       </c>
       <c r="B26" t="s" s="0">
-        <v>480</v>
+        <v>495</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="0">
-        <v>481</v>
+        <v>496</v>
       </c>
       <c r="B27" t="s" s="0">
-        <v>482</v>
+        <v>497</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="0">
-        <v>483</v>
+        <v>498</v>
       </c>
       <c r="B28" t="s" s="0">
-        <v>484</v>
+        <v>499</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="0">
-        <v>485</v>
+        <v>500</v>
       </c>
       <c r="B29" t="s" s="0">
-        <v>486</v>
+        <v>501</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="0">
-        <v>487</v>
+        <v>502</v>
       </c>
       <c r="B30" t="s" s="0">
-        <v>488</v>
+        <v>503</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="0">
-        <v>489</v>
+        <v>504</v>
       </c>
       <c r="B31" t="s" s="0">
-        <v>490</v>
+        <v>505</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s" s="0">
+        <v>506</v>
+      </c>
+      <c r="B32" t="s" s="0">
+        <v>507</v>
       </c>
     </row>
   </sheetData>
@@ -2465,12 +2524,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>156</v>
+        <v>160</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
   </sheetData>
@@ -2491,30 +2550,30 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>499</v>
+        <v>516</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>500</v>
+        <v>517</v>
       </c>
       <c r="C1" t="s" s="0">
-        <v>502</v>
+        <v>519</v>
       </c>
       <c r="D1" t="s" s="0">
-        <v>504</v>
+        <v>521</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>70</v>
+        <v>44</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>501</v>
+        <v>518</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>503</v>
+        <v>520</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>505</v>
+        <v>522</v>
       </c>
     </row>
   </sheetData>
@@ -2524,7 +2583,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B57"/>
+  <dimension ref="A1:B59"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -2981,6 +3040,22 @@
       </c>
       <c r="B57" t="s" s="0">
         <v>117</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="s" s="0">
+        <v>118</v>
+      </c>
+      <c r="B58" t="s" s="0">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="s" s="0">
+        <v>120</v>
+      </c>
+      <c r="B59" t="s" s="0">
+        <v>121</v>
       </c>
     </row>
   </sheetData>
@@ -2995,146 +3070,146 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>120</v>
+        <v>124</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>122</v>
+        <v>126</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>124</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>126</v>
+        <v>130</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>128</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>132</v>
+        <v>136</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>134</v>
+        <v>138</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>136</v>
+        <v>140</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>138</v>
+        <v>142</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>140</v>
+        <v>144</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>142</v>
+        <v>146</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>144</v>
+        <v>148</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>146</v>
+        <v>150</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>148</v>
+        <v>152</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>150</v>
+        <v>154</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>152</v>
+        <v>156</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>154</v>
+        <v>158</v>
       </c>
     </row>
   </sheetData>
@@ -3149,12 +3224,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>156</v>
+        <v>160</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
   </sheetData>
@@ -3164,271 +3239,287 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B33"/>
+  <dimension ref="A1:B35"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>160</v>
+        <v>164</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>161</v>
+        <v>92</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>162</v>
+        <v>165</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>164</v>
+        <v>167</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>166</v>
+        <v>169</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>168</v>
+        <v>171</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>170</v>
+        <v>173</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>172</v>
+        <v>175</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>174</v>
+        <v>177</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>176</v>
+        <v>179</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>178</v>
+        <v>181</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>180</v>
+        <v>183</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>186</v>
+        <v>189</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>188</v>
+        <v>191</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>190</v>
+        <v>193</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>192</v>
+        <v>195</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>194</v>
+        <v>197</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>196</v>
+        <v>199</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="0">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B20" t="s" s="0">
-        <v>198</v>
+        <v>201</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="0">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="B21" t="s" s="0">
-        <v>200</v>
+        <v>203</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="B22" t="s" s="0">
-        <v>202</v>
+        <v>205</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>204</v>
+        <v>207</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="0">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B24" t="s" s="0">
-        <v>206</v>
+        <v>209</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="0">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="B25" t="s" s="0">
-        <v>208</v>
+        <v>211</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="0">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="B26" t="s" s="0">
-        <v>210</v>
+        <v>213</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="0">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="B27" t="s" s="0">
-        <v>212</v>
+        <v>215</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="0">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="B28" t="s" s="0">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="0">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="B29" t="s" s="0">
-        <v>216</v>
+        <v>219</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="0">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="B30" t="s" s="0">
-        <v>218</v>
+        <v>221</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="0">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="B31" t="s" s="0">
-        <v>220</v>
+        <v>223</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s" s="0">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="B32" t="s" s="0">
-        <v>222</v>
+        <v>225</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s" s="0">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="B33" t="s" s="0">
-        <v>224</v>
+        <v>227</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="B34" t="s" s="0">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s" s="0">
+        <v>230</v>
+      </c>
+      <c r="B35" t="s" s="0">
+        <v>231</v>
       </c>
     </row>
   </sheetData>
@@ -3438,703 +3529,735 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B87"/>
+  <dimension ref="A1:B91"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>226</v>
+        <v>163</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>227</v>
+        <v>164</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>229</v>
+        <v>234</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>231</v>
+        <v>236</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>233</v>
+        <v>238</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>235</v>
+        <v>240</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>237</v>
+        <v>242</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>239</v>
+        <v>244</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>241</v>
+        <v>246</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>243</v>
+        <v>248</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>245</v>
+        <v>250</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>247</v>
+        <v>252</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>249</v>
+        <v>254</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>251</v>
+        <v>256</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>253</v>
+        <v>258</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>255</v>
+        <v>260</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>257</v>
+        <v>262</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>259</v>
+        <v>264</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>261</v>
+        <v>266</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>263</v>
+        <v>268</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="0">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="B20" t="s" s="0">
-        <v>265</v>
+        <v>270</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="0">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="B21" t="s" s="0">
-        <v>267</v>
+        <v>272</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="B22" t="s" s="0">
-        <v>269</v>
+        <v>274</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>271</v>
+        <v>276</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="0">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="B24" t="s" s="0">
-        <v>273</v>
+        <v>278</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="0">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="B25" t="s" s="0">
-        <v>275</v>
+        <v>280</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="0">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="B26" t="s" s="0">
-        <v>277</v>
+        <v>282</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="0">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="B27" t="s" s="0">
-        <v>279</v>
+        <v>284</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="0">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="B28" t="s" s="0">
-        <v>281</v>
+        <v>286</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="0">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="B29" t="s" s="0">
-        <v>283</v>
+        <v>288</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="0">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="B30" t="s" s="0">
-        <v>285</v>
+        <v>290</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="0">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="B31" t="s" s="0">
-        <v>287</v>
+        <v>292</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s" s="0">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="B32" t="s" s="0">
-        <v>289</v>
+        <v>294</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s" s="0">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="B33" t="s" s="0">
-        <v>291</v>
+        <v>296</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s" s="0">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="B34" t="s" s="0">
-        <v>293</v>
+        <v>298</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="0">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="B35" t="s" s="0">
-        <v>295</v>
+        <v>300</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="0">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="B36" t="s" s="0">
-        <v>297</v>
+        <v>302</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s" s="0">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="B37" t="s" s="0">
-        <v>299</v>
+        <v>304</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s" s="0">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="B38" t="s" s="0">
-        <v>301</v>
+        <v>306</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s" s="0">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="B39" t="s" s="0">
-        <v>303</v>
+        <v>308</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s" s="0">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="B40" t="s" s="0">
-        <v>305</v>
+        <v>310</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="0">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="B41" t="s" s="0">
-        <v>307</v>
+        <v>312</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="0">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="B42" t="s" s="0">
-        <v>309</v>
+        <v>314</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s" s="0">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="B43" t="s" s="0">
-        <v>311</v>
+        <v>316</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s" s="0">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="B44" t="s" s="0">
-        <v>313</v>
+        <v>318</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s" s="0">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="B45" t="s" s="0">
-        <v>315</v>
+        <v>320</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s" s="0">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="B46" t="s" s="0">
-        <v>317</v>
+        <v>322</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s" s="0">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="B47" t="s" s="0">
-        <v>319</v>
+        <v>324</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s" s="0">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="B48" t="s" s="0">
-        <v>321</v>
+        <v>326</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s" s="0">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="B49" t="s" s="0">
-        <v>323</v>
+        <v>328</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s" s="0">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="B50" t="s" s="0">
-        <v>325</v>
+        <v>330</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s" s="0">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="B51" t="s" s="0">
-        <v>327</v>
+        <v>332</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s" s="0">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="B52" t="s" s="0">
-        <v>329</v>
+        <v>334</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s" s="0">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="B53" t="s" s="0">
-        <v>331</v>
+        <v>336</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s" s="0">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="B54" t="s" s="0">
-        <v>333</v>
+        <v>338</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s" s="0">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="B55" t="s" s="0">
-        <v>335</v>
+        <v>340</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s" s="0">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="B56" t="s" s="0">
-        <v>337</v>
+        <v>342</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s" s="0">
-        <v>338</v>
+        <v>343</v>
       </c>
       <c r="B57" t="s" s="0">
-        <v>339</v>
+        <v>344</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s" s="0">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="B58" t="s" s="0">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s" s="0">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="B59" t="s" s="0">
-        <v>343</v>
+        <v>348</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="s" s="0">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="B60" t="s" s="0">
-        <v>345</v>
+        <v>350</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="s" s="0">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="B61" t="s" s="0">
-        <v>347</v>
+        <v>352</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="s" s="0">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="B62" t="s" s="0">
-        <v>349</v>
+        <v>354</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="s" s="0">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="B63" t="s" s="0">
-        <v>351</v>
+        <v>356</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="s" s="0">
-        <v>352</v>
+        <v>357</v>
       </c>
       <c r="B64" t="s" s="0">
-        <v>353</v>
+        <v>358</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="s" s="0">
-        <v>354</v>
+        <v>359</v>
       </c>
       <c r="B65" t="s" s="0">
-        <v>355</v>
+        <v>360</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="s" s="0">
-        <v>356</v>
+        <v>361</v>
       </c>
       <c r="B66" t="s" s="0">
-        <v>357</v>
+        <v>362</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="s" s="0">
-        <v>76</v>
+        <v>363</v>
       </c>
       <c r="B67" t="s" s="0">
-        <v>358</v>
+        <v>364</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="s" s="0">
-        <v>359</v>
+        <v>365</v>
       </c>
       <c r="B68" t="s" s="0">
-        <v>360</v>
+        <v>366</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="s" s="0">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="B69" t="s" s="0">
-        <v>362</v>
+        <v>368</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="s" s="0">
-        <v>363</v>
+        <v>369</v>
       </c>
       <c r="B70" t="s" s="0">
-        <v>364</v>
+        <v>370</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="s" s="0">
-        <v>191</v>
+        <v>371</v>
       </c>
       <c r="B71" t="s" s="0">
-        <v>192</v>
+        <v>372</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="s" s="0">
-        <v>365</v>
+        <v>373</v>
       </c>
       <c r="B72" t="s" s="0">
-        <v>366</v>
+        <v>374</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="s" s="0">
-        <v>367</v>
+        <v>375</v>
       </c>
       <c r="B73" t="s" s="0">
-        <v>368</v>
+        <v>376</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="s" s="0">
-        <v>369</v>
+        <v>377</v>
       </c>
       <c r="B74" t="s" s="0">
-        <v>370</v>
+        <v>378</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="s" s="0">
-        <v>371</v>
+        <v>379</v>
       </c>
       <c r="B75" t="s" s="0">
-        <v>372</v>
+        <v>380</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="s" s="0">
-        <v>373</v>
+        <v>381</v>
       </c>
       <c r="B76" t="s" s="0">
-        <v>374</v>
+        <v>382</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="s" s="0">
-        <v>375</v>
+        <v>383</v>
       </c>
       <c r="B77" t="s" s="0">
-        <v>376</v>
+        <v>384</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="s" s="0">
-        <v>377</v>
+        <v>385</v>
       </c>
       <c r="B78" t="s" s="0">
-        <v>378</v>
+        <v>386</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="s" s="0">
-        <v>379</v>
+        <v>4</v>
       </c>
       <c r="B79" t="s" s="0">
-        <v>380</v>
+        <v>387</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="s" s="0">
-        <v>381</v>
+        <v>388</v>
       </c>
       <c r="B80" t="s" s="0">
-        <v>382</v>
+        <v>389</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="s" s="0">
-        <v>383</v>
+        <v>390</v>
       </c>
       <c r="B81" t="s" s="0">
-        <v>384</v>
+        <v>391</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="s" s="0">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="B82" t="s" s="0">
-        <v>386</v>
+        <v>393</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="s" s="0">
-        <v>387</v>
+        <v>394</v>
       </c>
       <c r="B83" t="s" s="0">
-        <v>388</v>
+        <v>395</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="s" s="0">
-        <v>389</v>
+        <v>396</v>
       </c>
       <c r="B84" t="s" s="0">
-        <v>390</v>
+        <v>397</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="s" s="0">
-        <v>391</v>
+        <v>398</v>
       </c>
       <c r="B85" t="s" s="0">
-        <v>392</v>
+        <v>399</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="s" s="0">
-        <v>393</v>
+        <v>400</v>
       </c>
       <c r="B86" t="s" s="0">
-        <v>394</v>
+        <v>401</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="s" s="0">
-        <v>395</v>
+        <v>402</v>
       </c>
       <c r="B87" t="s" s="0">
-        <v>396</v>
+        <v>403</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="s" s="0">
+        <v>404</v>
+      </c>
+      <c r="B88" t="s" s="0">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="s" s="0">
+        <v>406</v>
+      </c>
+      <c r="B89" t="s" s="0">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="s" s="0">
+        <v>408</v>
+      </c>
+      <c r="B90" t="s" s="0">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="s" s="0">
+        <v>410</v>
+      </c>
+      <c r="B91" t="s" s="0">
+        <v>411</v>
       </c>
     </row>
   </sheetData>
@@ -4149,42 +4272,42 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>399</v>
+        <v>414</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>400</v>
+        <v>415</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>401</v>
+        <v>416</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>402</v>
+        <v>417</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>403</v>
+        <v>418</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>404</v>
+        <v>419</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>405</v>
+        <v>420</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>406</v>
+        <v>421</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>407</v>
+        <v>422</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>408</v>
+        <v>423</v>
       </c>
     </row>
   </sheetData>
@@ -4199,26 +4322,26 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>401</v>
+        <v>418</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>402</v>
+        <v>419</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>403</v>
+        <v>420</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>404</v>
+        <v>421</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>405</v>
+        <v>422</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>406</v>
+        <v>423</v>
       </c>
     </row>
   </sheetData>
@@ -4233,18 +4356,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>415</v>
+        <v>430</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>416</v>
+        <v>431</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>417</v>
+        <v>432</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>418</v>
+        <v>433</v>
       </c>
     </row>
   </sheetData>

</xml_diff>